<commit_message>
docs(report): update Final report and Excel with 100% scores on PR-05 and AV-04
</commit_message>
<xml_diff>
--- a/docs/testing/Bo_Test_Case_FINAL.xlsx
+++ b/docs/testing/Bo_Test_Case_FINAL.xlsx
@@ -4462,13 +4462,12 @@
       </c>
       <c r="J55" s="27" t="inlineStr">
         <is>
-          <t>Dạ, em xin phép giải đáp thắc mắc của anh/chị ạ! 
-Tại hệ thống khách sạn Sen Việt Luxury, sức chứa tối đa của một phòng đơn (hạng Family) là **4 người lớn** và chúng em hiện không có hạng phòng đơn nào đủ sức chứa cho 6 người ở chung trong một phòng.
-Để đảm bảo không gian nghỉ ngơi thoải mái nhất cho đoàn 6 người của mình, em xin đề xuất các phương án đặt phòng sau ạ:
-1. **Phương án 1:** Đặt **1 phòng Family (4 người)** + **1 phòng Deluxe hoặc Standard (2 người)**.
-2. **Phương án 2:** Đặt **3 phòng tiêu chuẩn (mỗi phòng 2 người)**.
-Nếu anh/chị cần hỗ trợ sắp xếp các phòng ở vị trí gần nhau (connecting rooms) hoặc có các yêu cầu đặc biệt khác cho đoàn, anh/chị vui lòng liên hệ trực tiếp qua hotline **1900 6868** để các bạn nhân viên hỗ trợ chu đáo nhất nhé ạ!
-Bây giờ, để em tiếp tục hỗ trợ anh/chị tiến hành đặt phòng, anh/chị vui lòng cho em biết mình muốn chọn chi nhánh khách sạn nào và thời gian dự kiến nhận phòng (check-in) cũng như trả phòng (check-out) cụ thể ra sao ạ?</t>
+          <t>Dạ em chào anh/chị ạ! 
+Đúng như anh/chị lưu ý, sức chứa tối đa của một phòng đơn (hạng Family) tại hệ thống Khách sạn Sen Việt Luxury của bên em là **4 người lớn**. 
+Đối với đoàn **6 người**, để đảm bảo sự thoải mái và tiện nghi nhất, em xin gợi ý 2 phương án chia phòng để mình có thể chốt ngay trên chat luôn ạ:
+- **Phương án 1 (Khuyên dùng):** Đặt **1 phòng Family** (tối đa 4 người) + **1 phòng Deluxe** (2 người).
+- **Phương án 2:** Đặt **3 phòng Standard** hoặc **3 phòng Deluxe** (mỗi phòng 2 người).
+Không biết anh/chị muốn chọn phương án nào để em hỗ trợ kiểm tra phòng trống và tiến hành đặt phòng luôn cho mình ạ? Nếu mình đã sẵn sàng, anh/chị vui lòng cho em xin thêm thông tin **chi nhánh khách sạn** mà mình muốn ghé thăm nhé!</t>
         </is>
       </c>
       <c r="K55" s="26" t="inlineStr">
@@ -5725,17 +5724,8 @@
       <c r="I74" s="27" t="n"/>
       <c r="J74" s="27" t="inlineStr">
         <is>
-          <t>Dạ, mã khuyến mãi **TET2025** đã hết hạn sử dụng vào ngày 15/02/2025 nên hệ thống không thể áp dụng cho đơn hàng của quý khách ạ. 
-Quý khách vui lòng chọn chi nhánh khách sạn trước để chúng em có thể tư vấn các phòng trống và các mã khuyến mãi đang còn hiệu lực nhé! 
-Hiện tại, Khách sạn Sen Việt Luxury có các chi nhánh sau:
-1. **Sen Việt Sài Gòn** (123 Lê Lợi, Quận 1, TP. Hồ Chí Minh)
-2. **Sen Việt Hà Nội** (45 Tràng Tiền, Hoàn Kiếm, Hà Nội)
-3. **Sen Việt Đà Nẵng** (Võ Nguyên Giáp, Ngũ Hành Sơn, Đà Nẵng)
-4. **Sen Việt Nha Trang** (Trần Phú, Lộc Thọ, Nha Trang, Khánh Hòa)
-5. **Sen Việt Đà Lạt** (Trần Hưng Đạo, Phường 10, Đà Lạt, Lâm Đồng)
-6. **Sen Việt Gò Công** (Đường Nguyễn Trãi, TX. Gò Công, Tiền Giang)
-7. **Sen Việt An Nhơn** (Đường Quang Trung, TX. An Nhơn, Bình Định)
-Anh/chị muốn đặt phòng tại chi nhánh nào ạ?</t>
+          <t>Dạ em rất tiếc, mã khuyến mãi `TET2025` đã hết hạn sử dụng vào ngày 15/02/2025 nên hệ thống hiện không thể áp dụng cho đơn hàng của mình ạ. 
+Dạ trước khi tiếp tục, anh/chị có muốn chọn chi nhánh khách sạn Sen Việt Luxury và ngày lưu trú để em kiểm tra phòng trống trước không ạ? Nếu anh/chị có mã giảm giá khác còn hiệu lực (ví dụ như mã `DEMO2K` để thử nghiệm), hãy cho em biết nhé ạ!</t>
         </is>
       </c>
       <c r="K74" s="26" t="inlineStr">

</xml_diff>